<commit_message>
feat: add side-by-side tax base breakdowns to reconciliation results and reporting sheets
</commit_message>
<xml_diff>
--- a/data/02 Exceptions.xlsx
+++ b/data/02 Exceptions.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Missing in KRA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Amount Mismatch" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="VAT Mismatch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Multiple Issues" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -218,8 +219,33 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_vat_mismatch" displayName="tbl_vat_mismatch" ref="A1:P25" headerRowCount="1">
-  <autoFilter ref="A1:P25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_vat_mismatch" displayName="tbl_vat_mismatch" ref="A1:P21" headerRowCount="1">
+  <autoFilter ref="A1:P21"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="CU Number"/>
+    <tableColumn id="2" name="Invoice Type"/>
+    <tableColumn id="3" name="Amount Match"/>
+    <tableColumn id="4" name="VAT Breakdown Match"/>
+    <tableColumn id="5" name="ERP PIN"/>
+    <tableColumn id="6" name="ERP Partner"/>
+    <tableColumn id="7" name="ERP Invoice #"/>
+    <tableColumn id="8" name="ERP Date"/>
+    <tableColumn id="9" name="ERP Amount"/>
+    <tableColumn id="10" name="ERP VAT"/>
+    <tableColumn id="11" name="KRA PIN"/>
+    <tableColumn id="12" name="KRA Partner"/>
+    <tableColumn id="13" name="KRA Invoice #"/>
+    <tableColumn id="14" name="KRA Date"/>
+    <tableColumn id="15" name="KRA Amount"/>
+    <tableColumn id="16" name="KRA VAT"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_multiple_issues" displayName="tbl_multiple_issues" ref="A1:P5" headerRowCount="1">
+  <autoFilter ref="A1:P5"/>
   <tableColumns count="16">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
@@ -1930,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2258,7 +2284,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>0040076780000820928</t>
+          <t>0040807450001963198</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2284,7 +2310,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>0040076780000820928</t>
+          <t>0040807450001963198</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -2293,7 +2319,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>4127.97</v>
+        <v>3304.69</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -2312,7 +2338,7 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>0040076780000820926</t>
+          <t>0040807450001963198</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -2321,7 +2347,7 @@
         </is>
       </c>
       <c r="O5" s="5" t="n">
-        <v>4127.94</v>
+        <v>3304.69</v>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -2332,12 +2358,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>0040805600001427233</t>
+          <t>0110371080000071470</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Mixed Tax</t>
+          <t>Single Tax</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2353,12 +2379,12 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>NAIVAS LIMITED</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>0040805600001427233</t>
+          <t>0110371080000071470</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -2367,7 +2393,7 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v>7657.07</v>
+        <v>2777.78</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
@@ -2376,17 +2402,17 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>P051123223G</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Naivas Limited</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>0040807450001427233</t>
+          <t>0110371080000071470</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -2395,18 +2421,18 @@
         </is>
       </c>
       <c r="O6" s="5" t="n">
-        <v>7657.06</v>
+        <v>2777.78</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>0, 16, EXEMPT</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>0040805600001555990</t>
+          <t>0110371080000071544</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2427,12 +2453,12 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>NAIVAS LIMITED</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>0040805600001555990</t>
+          <t>0110371080000071544</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -2441,7 +2467,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>3480</v>
+        <v>1388.89</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -2450,17 +2476,17 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>P051123223G</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Naivas Limited</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>0040805630001555990</t>
+          <t>0110371080000071544</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -2469,23 +2495,23 @@
         </is>
       </c>
       <c r="O7" s="5" t="n">
-        <v>3480</v>
+        <v>1388.89</v>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>0040807450001963198</t>
+          <t>0110371080000071898</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Mixed Tax</t>
+          <t>Single Tax</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2501,12 +2527,12 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>NAIVAS LIMITED</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>0040807450001963198</t>
+          <t>0110371080000071898</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -2515,7 +2541,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3304.69</v>
+        <v>3703.7</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -2524,17 +2550,17 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>P051123223G</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Naivas Limited</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>0040807450001963198</t>
+          <t>0110371080000071898</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -2543,18 +2569,18 @@
         </is>
       </c>
       <c r="O8" s="5" t="n">
-        <v>3304.69</v>
+        <v>3703.7</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>0, 16</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>0110371080000071470</t>
+          <t>0110371080000072019</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2580,7 +2606,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071470</t>
+          <t>0110371080000072019</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -2589,7 +2615,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v>2777.78</v>
+        <v>2314.81</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -2608,7 +2634,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071470</t>
+          <t>0110371080000072019</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -2617,7 +2643,7 @@
         </is>
       </c>
       <c r="O9" s="5" t="n">
-        <v>2777.78</v>
+        <v>2314.81</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -2628,7 +2654,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>0110371080000071544</t>
+          <t>0110396110000612860</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2649,12 +2675,12 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>VIVO ENERGY KENYA</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071544</t>
+          <t>0110396110000612860</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -2663,7 +2689,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="n">
-        <v>1388.89</v>
+        <v>14630.56</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -2672,17 +2698,17 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>P051199483R</t>
+          <t>P000591167T</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>VIVO ENERGY KENYA LIMITED</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071544</t>
+          <t>0110396110000612860</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -2691,7 +2717,7 @@
         </is>
       </c>
       <c r="O10" s="5" t="n">
-        <v>1388.89</v>
+        <v>14630.56</v>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
@@ -2702,7 +2728,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>0110371080000071898</t>
+          <t>0170939520000029944</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2723,12 +2749,12 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>Zm Petroleum Limited</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071898</t>
+          <t>0170939520000029944</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -2737,7 +2763,7 @@
         </is>
       </c>
       <c r="I11" s="5" t="n">
-        <v>3703.7</v>
+        <v>2777.78</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -2746,17 +2772,17 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>P051199483R</t>
+          <t>P051432685I</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>Zm Petroleum Limited</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>0110371080000071898</t>
+          <t>0170939520000029944</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -2765,7 +2791,7 @@
         </is>
       </c>
       <c r="O11" s="5" t="n">
-        <v>3703.7</v>
+        <v>2777.78</v>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
@@ -2776,7 +2802,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>0110371080000072019</t>
+          <t>0311143410000133206</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2797,12 +2823,12 @@
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>PREMIUM FUELS KENYA LIMITED</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>0110371080000072019</t>
+          <t>0311143410000133206</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -2811,7 +2837,7 @@
         </is>
       </c>
       <c r="I12" s="5" t="n">
-        <v>2314.81</v>
+        <v>8851.85</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
@@ -2820,17 +2846,17 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>P051199483R</t>
+          <t>P051450459C</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>MASCOT PETROLEUM</t>
+          <t>Premium Fuels Kenya Limited</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>0110371080000072019</t>
+          <t>0311143410000133206</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -2839,7 +2865,7 @@
         </is>
       </c>
       <c r="O12" s="5" t="n">
-        <v>2314.81</v>
+        <v>8851.85</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
@@ -2850,7 +2876,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>0110385140000039570</t>
+          <t>KRACU0300005514/424966</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2871,12 +2897,12 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>KINGS OIL INVESTMENTS LTD</t>
+          <t>LALJI RAMJI FILLING STATION LIMITED</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>0110385140000039570</t>
+          <t>KRACU0300005514/424966</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -2885,7 +2911,7 @@
         </is>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1851.85</v>
+        <v>3703.7</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
@@ -2894,17 +2920,17 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>P051502684I</t>
+          <t>P051318387R</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>KINGS OIL INVESTMENTS LIMITED</t>
+          <t>LALJI RAMJI FILLING STATION LIMITED</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>0110387540000039570</t>
+          <t>KRACU0300005514/424966</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -2913,7 +2939,7 @@
         </is>
       </c>
       <c r="O13" s="5" t="n">
-        <v>1851.85</v>
+        <v>3703.7</v>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
@@ -2924,7 +2950,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>0110396110000612860</t>
+          <t>KRACU0300007339/175927</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2945,12 +2971,12 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>VIVO ENERGY KENYA</t>
+          <t>SEA ANGEL SERVICES STATION LTD</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>0110396110000612860</t>
+          <t>KRACU0300007339/175927</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -2959,7 +2985,7 @@
         </is>
       </c>
       <c r="I14" s="5" t="n">
-        <v>14630.56</v>
+        <v>1851.85</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -2968,17 +2994,17 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>P000591167T</t>
+          <t>P051155776J</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>VIVO ENERGY KENYA LIMITED</t>
+          <t>Sea Angel Service Station Limited</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>0110396110000612860</t>
+          <t>KRACU0300007339/175927</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -2987,7 +3013,7 @@
         </is>
       </c>
       <c r="O14" s="5" t="n">
-        <v>14630.56</v>
+        <v>1851.85</v>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -2998,7 +3024,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>0170939520000029944</t>
+          <t>KRACU0300007646/70760</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -3019,12 +3045,12 @@
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Zm Petroleum Limited</t>
+          <t>FURQAN PETROLEUM LIMITED</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>0170939520000029944</t>
+          <t>KRACU0300007646/70760</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -3033,7 +3059,7 @@
         </is>
       </c>
       <c r="I15" s="5" t="n">
-        <v>2777.78</v>
+        <v>2314.81</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
@@ -3042,17 +3068,17 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>P051432685I</t>
+          <t>P051695568A</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Zm Petroleum Limited</t>
+          <t>Furqan Petroleum Limited</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>0170939520000029944</t>
+          <t>KRACU0300007646/70760</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -3061,7 +3087,7 @@
         </is>
       </c>
       <c r="O15" s="5" t="n">
-        <v>2777.78</v>
+        <v>2314.81</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
@@ -3072,7 +3098,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>0311143410000133206</t>
+          <t>KRACU0300007646/84382</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -3093,12 +3119,12 @@
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>PREMIUM FUELS KENYA LIMITED</t>
+          <t>FURQAN PETROLEUM LIMITED</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>0311143410000133206</t>
+          <t>KRACU0300007646/84382</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -3107,7 +3133,7 @@
         </is>
       </c>
       <c r="I16" s="5" t="n">
-        <v>8851.85</v>
+        <v>2314.81</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
@@ -3116,17 +3142,17 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>P051450459C</t>
+          <t>P051695568A</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Premium Fuels Kenya Limited</t>
+          <t>Furqan Petroleum Limited</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>0311143410000133206</t>
+          <t>KRACU0300007646/84382</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
@@ -3135,7 +3161,7 @@
         </is>
       </c>
       <c r="O16" s="5" t="n">
-        <v>8851.85</v>
+        <v>2314.81</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
@@ -3146,7 +3172,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>KRACU0300005514/424966</t>
+          <t>KRACU0300008829/10954</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -3167,12 +3193,12 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>LALJI RAMJI FILLING STATION LIMITED</t>
+          <t>PURE JOY VENTURES LTD</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300005514/424966</t>
+          <t>KRACU0300008829/10954</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -3181,7 +3207,7 @@
         </is>
       </c>
       <c r="I17" s="5" t="n">
-        <v>3703.7</v>
+        <v>2776.21</v>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
@@ -3190,17 +3216,17 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>P051318387R</t>
+          <t>P051621767H</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>LALJI RAMJI FILLING STATION LIMITED</t>
+          <t>Pure Joy Ventures Ltd</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300005514/424966</t>
+          <t>KRACU0300008829/10954</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -3209,7 +3235,7 @@
         </is>
       </c>
       <c r="O17" s="5" t="n">
-        <v>3703.7</v>
+        <v>2776.21</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
@@ -3220,7 +3246,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>KRACU0300007339/175927</t>
+          <t>KRACU0300009743/35400</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -3241,12 +3267,12 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>SEA ANGEL SERVICES STATION LTD</t>
+          <t>PIUS MBUVI MUNYASYA</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007339/175927</t>
+          <t>KRACU0300009743/35400</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -3255,7 +3281,7 @@
         </is>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1851.85</v>
+        <v>1852.35</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
@@ -3264,17 +3290,17 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>P051155776J</t>
+          <t>A002390054I</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>Sea Angel Service Station Limited</t>
+          <t>PIUS  MBUVI MUNYASYA</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007339/175927</t>
+          <t>KRACU0300009743/35400</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -3283,7 +3309,7 @@
         </is>
       </c>
       <c r="O18" s="5" t="n">
-        <v>1851.85</v>
+        <v>1852.35</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
@@ -3294,7 +3320,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>KRACU0300007646/70760</t>
+          <t>KRACU0300010725/11886</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -3315,12 +3341,12 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>FURQAN PETROLEUM LIMITED</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007646/70760</t>
+          <t>KRACU0300010725/11886</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -3329,7 +3355,7 @@
         </is>
       </c>
       <c r="I19" s="5" t="n">
-        <v>2314.81</v>
+        <v>1388.89</v>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
@@ -3338,17 +3364,17 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>P051695568A</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Furqan Petroleum Limited</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007646/70760</t>
+          <t>KRACU0300010725/11886</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -3357,7 +3383,7 @@
         </is>
       </c>
       <c r="O19" s="5" t="n">
-        <v>2314.81</v>
+        <v>1388.89</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
@@ -3368,7 +3394,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>KRACU0300007646/84382</t>
+          <t>KRACU0300010725/13232</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -3389,12 +3415,12 @@
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>FURQAN PETROLEUM LIMITED</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007646/84382</t>
+          <t>KRACU0300010725/13232</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -3403,7 +3429,7 @@
         </is>
       </c>
       <c r="I20" s="5" t="n">
-        <v>2314.81</v>
+        <v>1388.89</v>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
@@ -3412,17 +3438,17 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>P051695568A</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Furqan Petroleum Limited</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300007646/84382</t>
+          <t>KRACU0300010725/13232</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -3431,7 +3457,7 @@
         </is>
       </c>
       <c r="O20" s="5" t="n">
-        <v>2314.81</v>
+        <v>1388.89</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
@@ -3442,7 +3468,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>KRACU0300008829/10954</t>
+          <t>KRACU0300010725/22758</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -3463,12 +3489,12 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>PURE JOY VENTURES LTD</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300008829/10954</t>
+          <t>KRACU0300010725/22758</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -3477,7 +3503,7 @@
         </is>
       </c>
       <c r="I21" s="5" t="n">
-        <v>2776.21</v>
+        <v>1388.89</v>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
@@ -3486,17 +3512,17 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>P051621767H</t>
+          <t>P051199483R</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Pure Joy Ventures Ltd</t>
+          <t>MASCOT PETROLEUM</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>KRACU0300008829/10954</t>
+          <t>KRACU0300010725/22758</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -3505,7 +3531,7 @@
         </is>
       </c>
       <c r="O21" s="5" t="n">
-        <v>2776.21</v>
+        <v>1388.89</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
@@ -3513,297 +3539,414 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>KRACU0300009743/35400</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CU Number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Invoice Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Amount Match</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>VAT Breakdown Match</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ERP PIN</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Partner</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Invoice #</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Amount</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ERP VAT</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>KRA PIN</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Partner</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Invoice #</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Date</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Amount</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>KRA VAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>0040076780000820928</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Mixed Tax</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>NAIVAS LIMITED</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>0040076780000820928</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>4127.97</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>P051123223G</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Naivas Limited</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>0040076780000820926</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>4127.94</v>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>0, 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0040805600001427233</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mixed Tax</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NAIVAS LIMITED</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>0040805600001427233</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>7657.07</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>P051123223G</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Naivas Limited</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>0040807450001427233</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>7657.06</v>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>0, 16, EXEMPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>0040805600001555990</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Single Tax</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>PIUS MBUVI MUNYASYA</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300009743/35400</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>1852.35</v>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>A002390054I</t>
-        </is>
-      </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>PIUS  MBUVI MUNYASYA</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300009743/35400</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="n">
-        <v>1852.35</v>
-      </c>
-      <c r="P22" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/11886</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>NAIVAS LIMITED</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>0040805600001555990</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>3480</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>P051123223G</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Naivas Limited</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>0040805630001555990</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>3480</v>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0110385140000039570</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Single Tax</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/11886</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>P051199483R</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/11886</t>
-        </is>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="P23" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/13232</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Single Tax</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/13232</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>P051199483R</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/13232</t>
-        </is>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="P24" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/22758</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Single Tax</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/22758</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>P051199483R</t>
-        </is>
-      </c>
-      <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>MASCOT PETROLEUM</t>
-        </is>
-      </c>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>KRACU0300010725/22758</t>
-        </is>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O25" s="5" t="n">
-        <v>1388.89</v>
-      </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>KINGS OIL INVESTMENTS LTD</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>0110385140000039570</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>P051502684I</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>KINGS OIL INVESTMENTS LIMITED</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>0110387540000039570</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>

</xml_diff>

<commit_message>
feat: add new tax base columns to reconciliation results and update related schemas and exports
</commit_message>
<xml_diff>
--- a/data/02 Exceptions.xlsx
+++ b/data/02 Exceptions.xlsx
@@ -156,9 +156,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_missing_in_sap" displayName="tbl_missing_in_sap" ref="A1:J9" headerRowCount="1">
-  <autoFilter ref="A1:J9"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_missing_in_sap" displayName="tbl_missing_in_sap" ref="A1:N9" headerRowCount="1">
+  <autoFilter ref="A1:N9"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
     <tableColumn id="3" name="Amount Match"/>
@@ -169,15 +169,19 @@
     <tableColumn id="8" name="KRA Date"/>
     <tableColumn id="9" name="KRA Amount"/>
     <tableColumn id="10" name="KRA VAT"/>
+    <tableColumn id="11" name="KRA 16% Base"/>
+    <tableColumn id="12" name="KRA 8% Base"/>
+    <tableColumn id="13" name="KRA 0% Base"/>
+    <tableColumn id="14" name="KRA Exempt Base"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_missing_in_kra" displayName="tbl_missing_in_kra" ref="A1:J7" headerRowCount="1">
-  <autoFilter ref="A1:J7"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_missing_in_kra" displayName="tbl_missing_in_kra" ref="A1:N7" headerRowCount="1">
+  <autoFilter ref="A1:N7"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
     <tableColumn id="3" name="Amount Match"/>
@@ -188,15 +192,19 @@
     <tableColumn id="8" name="ERP Date"/>
     <tableColumn id="9" name="ERP Amount"/>
     <tableColumn id="10" name="ERP VAT"/>
+    <tableColumn id="11" name="ERP 16% Base"/>
+    <tableColumn id="12" name="ERP 8% Base"/>
+    <tableColumn id="13" name="ERP 0% Base"/>
+    <tableColumn id="14" name="ERP Exempt Base"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_amount_mismatch" displayName="tbl_amount_mismatch" ref="A1:P7" headerRowCount="1">
-  <autoFilter ref="A1:P7"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_amount_mismatch" displayName="tbl_amount_mismatch" ref="A1:X7" headerRowCount="1">
+  <autoFilter ref="A1:X7"/>
+  <tableColumns count="24">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
     <tableColumn id="3" name="Amount Match"/>
@@ -207,21 +215,29 @@
     <tableColumn id="8" name="ERP Date"/>
     <tableColumn id="9" name="ERP Amount"/>
     <tableColumn id="10" name="ERP VAT"/>
-    <tableColumn id="11" name="KRA PIN"/>
-    <tableColumn id="12" name="KRA Partner"/>
-    <tableColumn id="13" name="KRA Invoice #"/>
-    <tableColumn id="14" name="KRA Date"/>
-    <tableColumn id="15" name="KRA Amount"/>
-    <tableColumn id="16" name="KRA VAT"/>
+    <tableColumn id="11" name="ERP 16% Base"/>
+    <tableColumn id="12" name="ERP 8% Base"/>
+    <tableColumn id="13" name="ERP 0% Base"/>
+    <tableColumn id="14" name="ERP Exempt Base"/>
+    <tableColumn id="15" name="KRA PIN"/>
+    <tableColumn id="16" name="KRA Partner"/>
+    <tableColumn id="17" name="KRA Invoice #"/>
+    <tableColumn id="18" name="KRA Date"/>
+    <tableColumn id="19" name="KRA Amount"/>
+    <tableColumn id="20" name="KRA VAT"/>
+    <tableColumn id="21" name="KRA 16% Base"/>
+    <tableColumn id="22" name="KRA 8% Base"/>
+    <tableColumn id="23" name="KRA 0% Base"/>
+    <tableColumn id="24" name="KRA Exempt Base"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_vat_mismatch" displayName="tbl_vat_mismatch" ref="A1:P21" headerRowCount="1">
-  <autoFilter ref="A1:P21"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_vat_mismatch" displayName="tbl_vat_mismatch" ref="A1:X21" headerRowCount="1">
+  <autoFilter ref="A1:X21"/>
+  <tableColumns count="24">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
     <tableColumn id="3" name="Amount Match"/>
@@ -232,21 +248,29 @@
     <tableColumn id="8" name="ERP Date"/>
     <tableColumn id="9" name="ERP Amount"/>
     <tableColumn id="10" name="ERP VAT"/>
-    <tableColumn id="11" name="KRA PIN"/>
-    <tableColumn id="12" name="KRA Partner"/>
-    <tableColumn id="13" name="KRA Invoice #"/>
-    <tableColumn id="14" name="KRA Date"/>
-    <tableColumn id="15" name="KRA Amount"/>
-    <tableColumn id="16" name="KRA VAT"/>
+    <tableColumn id="11" name="ERP 16% Base"/>
+    <tableColumn id="12" name="ERP 8% Base"/>
+    <tableColumn id="13" name="ERP 0% Base"/>
+    <tableColumn id="14" name="ERP Exempt Base"/>
+    <tableColumn id="15" name="KRA PIN"/>
+    <tableColumn id="16" name="KRA Partner"/>
+    <tableColumn id="17" name="KRA Invoice #"/>
+    <tableColumn id="18" name="KRA Date"/>
+    <tableColumn id="19" name="KRA Amount"/>
+    <tableColumn id="20" name="KRA VAT"/>
+    <tableColumn id="21" name="KRA 16% Base"/>
+    <tableColumn id="22" name="KRA 8% Base"/>
+    <tableColumn id="23" name="KRA 0% Base"/>
+    <tableColumn id="24" name="KRA Exempt Base"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_multiple_issues" displayName="tbl_multiple_issues" ref="A1:P5" headerRowCount="1">
-  <autoFilter ref="A1:P5"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_multiple_issues" displayName="tbl_multiple_issues" ref="A1:X5" headerRowCount="1">
+  <autoFilter ref="A1:X5"/>
+  <tableColumns count="24">
     <tableColumn id="1" name="CU Number"/>
     <tableColumn id="2" name="Invoice Type"/>
     <tableColumn id="3" name="Amount Match"/>
@@ -257,12 +281,20 @@
     <tableColumn id="8" name="ERP Date"/>
     <tableColumn id="9" name="ERP Amount"/>
     <tableColumn id="10" name="ERP VAT"/>
-    <tableColumn id="11" name="KRA PIN"/>
-    <tableColumn id="12" name="KRA Partner"/>
-    <tableColumn id="13" name="KRA Invoice #"/>
-    <tableColumn id="14" name="KRA Date"/>
-    <tableColumn id="15" name="KRA Amount"/>
-    <tableColumn id="16" name="KRA VAT"/>
+    <tableColumn id="11" name="ERP 16% Base"/>
+    <tableColumn id="12" name="ERP 8% Base"/>
+    <tableColumn id="13" name="ERP 0% Base"/>
+    <tableColumn id="14" name="ERP Exempt Base"/>
+    <tableColumn id="15" name="KRA PIN"/>
+    <tableColumn id="16" name="KRA Partner"/>
+    <tableColumn id="17" name="KRA Invoice #"/>
+    <tableColumn id="18" name="KRA Date"/>
+    <tableColumn id="19" name="KRA Amount"/>
+    <tableColumn id="20" name="KRA VAT"/>
+    <tableColumn id="21" name="KRA 16% Base"/>
+    <tableColumn id="22" name="KRA 8% Base"/>
+    <tableColumn id="23" name="KRA 0% Base"/>
+    <tableColumn id="24" name="KRA Exempt Base"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -557,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -570,6 +602,10 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -623,6 +659,26 @@
           <t>KRA VAT</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 16% Base</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 8% Base</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 0% Base</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Exempt Base</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -637,12 +693,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -672,6 +728,18 @@
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>9584.91</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -687,12 +755,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -722,6 +790,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -737,12 +817,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -772,6 +852,18 @@
         <is>
           <t>EXEMPT</t>
         </is>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>-13561</v>
       </c>
     </row>
     <row r="5">
@@ -787,12 +879,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -822,6 +914,18 @@
         <is>
           <t>EXEMPT</t>
         </is>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>-5776</v>
       </c>
     </row>
     <row r="6">
@@ -837,12 +941,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -872,6 +976,18 @@
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>925.9299999999999</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -887,12 +1003,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -922,6 +1038,18 @@
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>462.96</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -937,12 +1065,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -972,6 +1100,18 @@
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>13888.88</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -987,12 +1127,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1022,6 +1162,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>2589.58</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1038,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1051,6 +1203,10 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1104,6 +1260,26 @@
           <t>ERP VAT</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 16% Base</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 8% Base</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 0% Base</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Exempt Base</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1118,12 +1294,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr"/>
@@ -1149,6 +1325,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>2157000</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1164,12 +1352,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
@@ -1195,6 +1383,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>27100</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1210,12 +1410,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
@@ -1241,6 +1441,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>14000</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1256,12 +1468,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
@@ -1287,6 +1499,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>8940</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1302,12 +1526,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
@@ -1333,6 +1557,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>120000</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1348,12 +1584,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
@@ -1379,6 +1615,18 @@
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>26000</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1395,7 +1643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1408,12 +1656,20 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1469,32 +1725,72 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>ERP 16% Base</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 8% Base</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 0% Base</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Exempt Base</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>KRA PIN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>KRA Partner</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>KRA Invoice #</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>KRA Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>KRA Amount</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>KRA VAT</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 16% Base</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 8% Base</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 0% Base</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Exempt Base</t>
         </is>
       </c>
     </row>
@@ -1543,33 +1839,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="5" t="n">
+        <v>32228.59</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>P000591096X</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Kenya Power &amp; Lighting Company Ltd</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>0020113710000346124</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="n">
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="n">
         <v>29265.08</v>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>29265.08</v>
+      </c>
+      <c r="V2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1617,33 +1937,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="5" t="n">
+        <v>4734.23</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>P000591096X</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Kenya Power &amp; Lighting Company Ltd</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>0020116570000390636</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="n">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="n">
         <v>4298.58</v>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>4298.58</v>
+      </c>
+      <c r="V3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1691,33 +2035,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="5" t="n">
+        <v>2359.83</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>P052032731M</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>FLAVOR TOWN CAFE KENYA LIMITED</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>0090973760000364781</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="n">
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="n">
         <v>2313.56</v>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="U4" s="5" t="n">
+        <v>2313.56</v>
+      </c>
+      <c r="V4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1765,33 +2133,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="5" t="n">
+        <v>2679.01</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>P051129820X</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Safaricom</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>7462187335086645119</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="n">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="n">
         <v>2678.88</v>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="U5" s="5" t="n">
+        <v>2678.88</v>
+      </c>
+      <c r="V5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1839,33 +2231,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="5" t="n">
+        <v>9482.76</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>P051326978T</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>AFRICASTALKING (K) LIMITED</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>KRACU0300001381/29013</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="n">
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="n">
         <v>9568.969999999999</v>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
+      </c>
+      <c r="U6" s="5" t="n">
+        <v>9568.969999999999</v>
+      </c>
+      <c r="V6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1913,33 +2329,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="5" t="n">
+        <v>2288</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>P051695568A</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Furqan Petroleum Limited</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>KRACU0300007646/83601</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="n">
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>2287.25</v>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>16, 8</t>
         </is>
+      </c>
+      <c r="U7" s="5" t="n">
+        <v>1362.07</v>
+      </c>
+      <c r="V7" s="5" t="n">
+        <v>925.1799999999999</v>
+      </c>
+      <c r="W7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1956,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1969,12 +2409,20 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2030,32 +2478,72 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>ERP 16% Base</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 8% Base</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 0% Base</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Exempt Base</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>KRA PIN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>KRA Partner</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>KRA Invoice #</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>KRA Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>KRA Amount</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>KRA VAT</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 16% Base</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 8% Base</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 0% Base</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Exempt Base</t>
         </is>
       </c>
     </row>
@@ -2104,33 +2592,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>A007129101F</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>ALEXANDER MWAKUNGU MWALUA</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>0020106030000359193</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="n">
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="n">
         <v>1851.85</v>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="W2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2178,33 +2690,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="5" t="n">
+        <v>2778.15</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>A007030914X</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>GERISHON MARK KIBAGENDI</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>0020106130000475731</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="n">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="n">
         <v>2778.15</v>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="5" t="n">
+        <v>2778.15</v>
+      </c>
+      <c r="W3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2252,33 +2788,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="5" t="n">
+        <v>5018.17</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>P051123223G</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Naivas Limited</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>0040076780000806904</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="n">
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="n">
         <v>5018.19</v>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>0, 16, EXEMPT</t>
         </is>
+      </c>
+      <c r="U4" s="5" t="n">
+        <v>2105.19</v>
+      </c>
+      <c r="V4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="5" t="n">
+        <v>2784</v>
+      </c>
+      <c r="X4" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="5">
@@ -2326,33 +2886,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="5" t="n">
+        <v>3304.69</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>P051123223G</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Naivas Limited</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>0040807450001963198</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="n">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="n">
         <v>3304.69</v>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>0, 16</t>
         </is>
+      </c>
+      <c r="U5" s="5" t="n">
+        <v>520.6900000000001</v>
+      </c>
+      <c r="V5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="5" t="n">
+        <v>2784</v>
+      </c>
+      <c r="X5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2400,33 +2984,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="5" t="n">
+        <v>2777.78</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>0110371080000071470</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="n">
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="n">
         <v>2777.78</v>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="5" t="n">
+        <v>2777.78</v>
+      </c>
+      <c r="W6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2474,33 +3082,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>0110371080000071544</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="n">
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>1388.89</v>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="W7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2548,33 +3180,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="5" t="n">
+        <v>3703.7</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>0110371080000071898</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="n">
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="n">
         <v>3703.7</v>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="5" t="n">
+        <v>3703.7</v>
+      </c>
+      <c r="W8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2622,33 +3278,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>0110371080000072019</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="n">
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="n">
         <v>2314.81</v>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="W9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2696,33 +3376,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="5" t="n">
+        <v>14630.56</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>P000591167T</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>VIVO ENERGY KENYA LIMITED</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>0110396110000612860</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="n">
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="n">
         <v>14630.56</v>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="5" t="n">
+        <v>14630.56</v>
+      </c>
+      <c r="W10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2770,33 +3474,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="5" t="n">
+        <v>2777.78</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>P051432685I</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>Zm Petroleum Limited</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>0170939520000029944</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="n">
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="n">
         <v>2777.78</v>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="5" t="n">
+        <v>2777.78</v>
+      </c>
+      <c r="W11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2844,33 +3572,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" s="5" t="n">
+        <v>8851.85</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>P051450459C</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>Premium Fuels Kenya Limited</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>0311143410000133206</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="n">
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="n">
         <v>8851.85</v>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="5" t="n">
+        <v>8851.85</v>
+      </c>
+      <c r="W12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2918,33 +3670,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" s="5" t="n">
+        <v>3703.7</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>P051318387R</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>LALJI RAMJI FILLING STATION LIMITED</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>KRACU0300005514/424966</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="n">
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="n">
         <v>3703.7</v>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="T13" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="5" t="n">
+        <v>3703.7</v>
+      </c>
+      <c r="W13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2992,33 +3768,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>P051155776J</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>Sea Angel Service Station Limited</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>KRACU0300007339/175927</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="n">
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="n">
         <v>1851.85</v>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="T14" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="W14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3066,33 +3866,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>P051695568A</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>Furqan Petroleum Limited</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>KRACU0300007646/70760</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="n">
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="n">
         <v>2314.81</v>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="T15" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="W15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3140,33 +3964,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>P051695568A</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>Furqan Petroleum Limited</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>KRACU0300007646/84382</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="n">
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="n">
         <v>2314.81</v>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="T16" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="5" t="n">
+        <v>2314.81</v>
+      </c>
+      <c r="W16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3214,33 +4062,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" s="5" t="n">
+        <v>2776.21</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>P051621767H</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>Pure Joy Ventures Ltd</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>KRACU0300008829/10954</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O17" s="5" t="n">
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="n">
         <v>2776.21</v>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="T17" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="5" t="n">
+        <v>2776.21</v>
+      </c>
+      <c r="W17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3288,33 +4160,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="5" t="n">
+        <v>1852.35</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>A002390054I</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>PIUS  MBUVI MUNYASYA</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>KRACU0300009743/35400</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="n">
+      <c r="R18" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="n">
         <v>1852.35</v>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="T18" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="5" t="n">
+        <v>1852.35</v>
+      </c>
+      <c r="W18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -3362,33 +4258,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>KRACU0300010725/11886</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="n">
+      <c r="R19" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="n">
         <v>1388.89</v>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="T19" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="W19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3436,33 +4356,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>KRACU0300010725/13232</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="n">
+      <c r="R20" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="n">
         <v>1388.89</v>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="T20" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="W20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3510,33 +4454,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>P051199483R</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="P21" s="3" t="inlineStr">
         <is>
           <t>MASCOT PETROLEUM</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="Q21" s="3" t="inlineStr">
         <is>
           <t>KRACU0300010725/22758</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="n">
+      <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="n">
         <v>1388.89</v>
       </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="T21" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="5" t="n">
+        <v>1388.89</v>
+      </c>
+      <c r="W21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3553,7 +4521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3566,12 +4534,20 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3627,32 +4603,72 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>ERP 16% Base</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 8% Base</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ERP 0% Base</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Exempt Base</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>KRA PIN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>KRA Partner</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>KRA Invoice #</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>KRA Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>KRA Amount</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>KRA VAT</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 16% Base</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 8% Base</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>KRA 0% Base</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>KRA Exempt Base</t>
         </is>
       </c>
     </row>
@@ -3701,33 +4717,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="5" t="n">
+        <v>4127.97</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>P051123223G</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Naivas Limited</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>0040076780000820926</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="n">
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="n">
         <v>4127.94</v>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>0, 16</t>
         </is>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>1343.94</v>
+      </c>
+      <c r="V2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="5" t="n">
+        <v>2784</v>
+      </c>
+      <c r="X2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3775,33 +4815,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="5" t="n">
+        <v>7657.07</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>P051123223G</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Naivas Limited</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>0040807450001427233</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="n">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="n">
         <v>7657.06</v>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>0, 16, EXEMPT</t>
         </is>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>6962.06</v>
+      </c>
+      <c r="V3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="5" t="n">
+        <v>395</v>
+      </c>
+      <c r="X3" s="5" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="4">
@@ -3849,33 +4913,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="5" t="n">
+        <v>3480</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>P051123223G</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Naivas Limited</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>0040805630001555990</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="n">
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="n">
         <v>3480</v>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
+      </c>
+      <c r="U4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="5" t="n">
+        <v>3480</v>
+      </c>
+      <c r="X4" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3923,33 +5011,57 @@
           <t>16</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>P051502684I</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>KINGS OIL INVESTMENTS LIMITED</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>0110387540000039570</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="n">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="n">
         <v>1851.85</v>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="U5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="5" t="n">
+        <v>1851.85</v>
+      </c>
+      <c r="W5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>